<commit_message>
Mise à jour 04/04/2025
Integration d'une prime de risque
Correction erreurs comptables sur le bloc auto (suppression de la double comptabilité des subventions et modification de l'équation CHM)
</commit_message>
<xml_diff>
--- a/data/calibrations/recalage parc immobilier_new2.xlsx
+++ b/data/calibrations/recalage parc immobilier_new2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\ThreeME\data\calibrations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C48172D-4BE4-4AD8-AEA9-FE5107050659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF7EE5A5-09EE-4B70-8E2B-795CA0E8AD65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{F3B8202A-200E-4C94-BB50-F6C7EC74A6D2}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{F3B8202A-200E-4C94-BB50-F6C7EC74A6D2}"/>
   </bookViews>
   <sheets>
     <sheet name="result" sheetId="1" r:id="rId1"/>
@@ -4384,7 +4384,13 @@
       <sheetData sheetId="21" refreshError="1"/>
       <sheetData sheetId="22" refreshError="1"/>
       <sheetData sheetId="23" refreshError="1"/>
-      <sheetData sheetId="24" refreshError="1"/>
+      <sheetData sheetId="24">
+        <row r="2">
+          <cell r="C2">
+            <v>0.99172610111270254</v>
+          </cell>
+        </row>
+      </sheetData>
       <sheetData sheetId="25">
         <row r="112">
           <cell r="C112">

</xml_diff>